<commit_message>
Revised 1st, 2nd floor to first, second floor
</commit_message>
<xml_diff>
--- a/UICLibraryData.xlsx
+++ b/UICLibraryData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Henry\Downloads\CS424_P1\Project-1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0A999F8-ADAD-470D-9D68-54248B6F9171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D867021A-8B8D-43AE-9C6E-BD0EC7DE4408}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4820" yWindow="2450" windowWidth="19200" windowHeight="11170" xr2:uid="{68D7DA14-3BBB-4245-B58F-0CCF1E067232}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{68D7DA14-3BBB-4245-B58F-0CCF1E067232}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -59,12 +59,6 @@
     <t>Lower than usual</t>
   </si>
   <si>
-    <t>1st</t>
-  </si>
-  <si>
-    <t>2nd</t>
-  </si>
-  <si>
     <t>occupancy_count</t>
   </si>
   <si>
@@ -126,6 +120,12 @@
   </si>
   <si>
     <t>285</t>
+  </si>
+  <si>
+    <t>first</t>
+  </si>
+  <si>
+    <t>second</t>
   </si>
 </sst>
 </file>
@@ -510,36 +510,36 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" t="s">
         <v>11</v>
       </c>
-      <c r="B1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C1" t="s">
-        <v>13</v>
-      </c>
       <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" t="s">
         <v>8</v>
-      </c>
-      <c r="E1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F1" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E2" t="s">
         <v>1</v>
@@ -547,16 +547,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
         <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E3" t="s">
         <v>2</v>
@@ -567,16 +567,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
         <v>0</v>
       </c>
       <c r="C4" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="E4" t="s">
         <v>1</v>
@@ -584,16 +584,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
         <v>0</v>
       </c>
       <c r="C5" t="s">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E5" t="s">
         <v>3</v>
@@ -604,16 +604,16 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
         <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E6" t="s">
         <v>1</v>
@@ -621,16 +621,16 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
         <v>0</v>
       </c>
       <c r="C7" t="s">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E7" t="s">
         <v>3</v>
@@ -641,16 +641,16 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
         <v>0</v>
       </c>
       <c r="C8" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E8" t="s">
         <v>1</v>
@@ -658,16 +658,16 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
         <v>0</v>
       </c>
       <c r="C9" t="s">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E9" t="s">
         <v>2</v>
@@ -678,16 +678,16 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B10" t="s">
         <v>0</v>
       </c>
       <c r="C10" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E10" t="s">
         <v>1</v>
@@ -698,16 +698,16 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B11" t="s">
         <v>0</v>
       </c>
       <c r="C11" t="s">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E11" t="s">
         <v>2</v>

</xml_diff>

<commit_message>
Upload sketch 02 and 03
</commit_message>
<xml_diff>
--- a/UICLibraryData.xlsx
+++ b/UICLibraryData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Henry\Downloads\CS424_P1\Project-1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D867021A-8B8D-43AE-9C6E-BD0EC7DE4408}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9849FB23-40FF-4535-B94D-16D145BEE4AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{68D7DA14-3BBB-4245-B58F-0CCF1E067232}"/>
   </bookViews>
@@ -559,7 +559,7 @@
         <v>18</v>
       </c>
       <c r="E3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3" t="s">
         <v>4</v>

</xml_diff>